<commit_message>
fix: resolve firebase-admin initialization conflict, ensure distinct PDF hashes in Pass 2, and successfully run report regeneration script
</commit_message>
<xml_diff>
--- a/artifacts/sample-v5/Verifier Workspace.xlsx
+++ b/artifacts/sample-v5/Verifier Workspace.xlsx
@@ -389,7 +389,7 @@
       </c>
       <c r="B10" s="11">
         <f>COUNTA(EVIDENCE!A2:A1048576)</f>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C10" t="inlineStr" s="4">
         <is>
@@ -397,7 +397,7 @@
         </is>
       </c>
       <c r="D10" s="8">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11">
@@ -1951,7 +1951,7 @@
       </c>
       <c r="C4" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">11111111-1111-4111-8111-111111111111</t>
+          <t xml:space="preserve">11111111-1111-4111-8111-222222222222</t>
         </is>
       </c>
       <c r="D4" t="inlineStr" s="5">
@@ -2647,7 +2647,7 @@
       </c>
       <c r="E2" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">11111111-1111-4111-8111-111111111111</t>
+          <t xml:space="preserve">11111111-1111-4111-8111-555555555555</t>
         </is>
       </c>
       <c r="F2" t="inlineStr" s="1">
@@ -2684,7 +2684,7 @@
       </c>
       <c r="E3" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">11111111-1111-4111-8111-111111111111</t>
+          <t xml:space="preserve">11111111-1111-4111-8111-333333333333</t>
         </is>
       </c>
       <c r="F3" t="inlineStr" s="1">
@@ -2721,7 +2721,7 @@
       </c>
       <c r="E4" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">11111111-1111-4111-8111-111111111111</t>
+          <t xml:space="preserve">11111111-1111-4111-8111-333333333333</t>
         </is>
       </c>
       <c r="F4" t="inlineStr" s="1">
@@ -2890,60 +2890,225 @@
     <row r="2">
       <c r="A2" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">11111111-1111-4111-8111-111111111111</t>
+          <t xml:space="preserve">11111111-1111-4111-8111-222222222222</t>
         </is>
       </c>
       <c r="B2" t="inlineStr" s="1">
         <is>
+          <t xml:space="preserve">CUSTOMS_DECLARATION</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">customs-declaration-classification.txt</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Customs Authority</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">2026-03-31</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">131f55d58925bbb16c2b5fc319042056ebcb0e5d192f642740fb7a0fa246bc7c</t>
+        </is>
+      </c>
+      <c r="G2" s="8">
+        <v>92</v>
+      </c>
+      <c r="H2" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">APPROVED</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">SUPPORTED</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">CLEAN</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">importerIdentity.eoriNumber | goods.0.cnCode | goods.1.cnCode | exporterIdentity.legalName | exporterIdentity.address | importerIdentity.legalName | importerIdentity.eoriNumber | installation.name | installation.country | installation.productionRoute | reportingPeriod.year | reportingPeriod.quarter | goods.0.cnCode | goods.0.allocationShare | goods.1.cnCode | goods.1.allocationShare</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">11111111-1111-4111-8111-333333333333</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">UTILITY_BILL</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">electricity-utility-invoice.txt</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">National Power Utility</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">2026-03-31</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">7e9c3cdb25683a0e8ce19c6c4f0c4048e2ef18fa76c94cbe122f4e82eeb5f335</t>
+        </is>
+      </c>
+      <c r="G3" s="8">
+        <v>106</v>
+      </c>
+      <c r="H3" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">APPROVED</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">SUPPORTED</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">CLEAN</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">electricityConsumed | gridEmissionFactor</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">11111111-1111-4111-8111-444444444444</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">PRODUCTION_RECONCILIATION_REPORT</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">production-reconciliation-ledger.txt</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Internal Production Auditor</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">2026-03-31</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">c5ecc502ccc8d7accbfb3302bbc20577301d605d967ed003e95a6056d79d6062</t>
+        </is>
+      </c>
+      <c r="G4" s="8">
+        <v>89</v>
+      </c>
+      <c r="H4" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">APPROVED</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">SUPPORTED</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">CLEAN</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">goods.0.productionVolume | goods.0.allocationShare | goods.1.productionVolume | goods.1.allocationShare</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">11111111-1111-4111-8111-555555555555</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr" s="1">
+        <is>
           <t xml:space="preserve">PRIMARY_MONITORING_AND_CUSTOMS_PACKAGE</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr" s="1">
+      <c r="C5" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">verified-monitoring-package.txt</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr" s="1">
+      <c r="D5" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Independent Monitoring Auditor</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr" s="1">
+      <c r="E5" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">2026-03-31</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr" s="1">
+      <c r="F5" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">52f88d25d5eba4319069b122447ad9073e41f2d4e7aafeede6bc99ccab29e634</t>
         </is>
       </c>
-      <c r="G2" s="8">
+      <c r="G5" s="8">
         <v>135</v>
       </c>
-      <c r="H2" t="inlineStr" s="1">
+      <c r="H5" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">APPROVED</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr" s="1">
+      <c r="I5" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">SUPPORTED</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr" s="1">
+      <c r="J5" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">CLEAN</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">importerIdentity.eoriNumber | goods.0.cnCode | goods.0.productionVolume | goods.0.allocationShare | goods.1.cnCode | goods.1.productionVolume | goods.1.allocationShare | directEmissions | electricityConsumed | gridEmissionFactor | exporterIdentity.legalName | exporterIdentity.address | importerIdentity.legalName | importerIdentity.eoriNumber | installation.name | installation.country | installation.productionRoute | reportingPeriod.year | reportingPeriod.quarter | goods.0.cnCode | goods.0.allocationShare | goods.1.cnCode | goods.1.allocationShare</t>
+      <c r="K5" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">directEmissions</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K2"/>
+  <autoFilter ref="A1:K5"/>
   <conditionalFormatting sqref="H2:H1048576">
     <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="PASS">
       <formula>NOT(ISERROR(SEARCH("PASS",H2)))</formula>
@@ -3064,7 +3229,7 @@
       </c>
       <c r="H2" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">11111111-1111-4111-8111-111111111111</t>
+          <t xml:space="preserve">11111111-1111-4111-8111-555555555555</t>
         </is>
       </c>
     </row>
@@ -3106,7 +3271,7 @@
       </c>
       <c r="H3" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">11111111-1111-4111-8111-111111111111</t>
+          <t xml:space="preserve">11111111-1111-4111-8111-444444444444</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3463,7 @@
       </c>
       <c r="D7" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">1 approved and clean evidence file(s)</t>
+          <t xml:space="preserve">4 approved and clean evidence file(s)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: resolve V4 Operator Report PDF test failures, type definitions and compliance rules
</commit_message>
<xml_diff>
--- a/artifacts/sample-v5/Verifier Workspace.xlsx
+++ b/artifacts/sample-v5/Verifier Workspace.xlsx
@@ -495,17 +495,17 @@
     <row r="2">
       <c r="A2" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">QC_00</t>
+          <t xml:space="preserve">QC_SCENARIO</t>
         </is>
       </c>
       <c r="B2" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Operator, installation and boundary identity</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">Illustrative scenario replacement</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">NOT_APPLICABLE</t>
         </is>
       </c>
       <c r="D2" t="inlineStr" s="1">
@@ -515,19 +515,19 @@
       </c>
       <c r="E2" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">REM_COMPLETE_CASE_IDENTITY</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">QC_01</t>
+          <t xml:space="preserve">QC_00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">EORI format and evidence</t>
+          <t xml:space="preserve">Operator, installation and boundary identity</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="5">
@@ -542,19 +542,19 @@
       </c>
       <c r="E3" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">REM_COMPLETE_CASE_IDENTITY</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">QC_02</t>
+          <t xml:space="preserve">QC_01</t>
         </is>
       </c>
       <c r="B4" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Definitive-period reporting year</t>
+          <t xml:space="preserve">EORI format and evidence</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="5">
@@ -569,19 +569,19 @@
       </c>
       <c r="E4" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">REM_CORRECT_REPORTING_YEAR</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">QC_03_0</t>
+          <t xml:space="preserve">QC_02</t>
         </is>
       </c>
       <c r="B5" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Good 1 CN code and evidence</t>
+          <t xml:space="preserve">Definitive-period reporting year</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="5">
@@ -596,19 +596,19 @@
       </c>
       <c r="E5" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">REM_CORRECT_REPORTING_YEAR</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">QC_04_0</t>
+          <t xml:space="preserve">QC_03_0</t>
         </is>
       </c>
       <c r="B6" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Good 1 production and evidence</t>
+          <t xml:space="preserve">Good 1 CN code and evidence</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="5">
@@ -630,12 +630,12 @@
     <row r="7">
       <c r="A7" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">QC_05_0</t>
+          <t xml:space="preserve">QC_04_0</t>
         </is>
       </c>
       <c r="B7" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Good 1 sector</t>
+          <t xml:space="preserve">Good 1 production and evidence</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="5">
@@ -650,19 +650,19 @@
       </c>
       <c r="E7" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">REM_SELECT_SUPPORTED_SECTOR</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">QC_03_1</t>
+          <t xml:space="preserve">QC_05_0</t>
         </is>
       </c>
       <c r="B8" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Good 2 CN code and evidence</t>
+          <t xml:space="preserve">Good 1 sector</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="5">
@@ -677,19 +677,19 @@
       </c>
       <c r="E8" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">REM_SELECT_SUPPORTED_SECTOR</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">QC_04_1</t>
+          <t xml:space="preserve">QC_03_1</t>
         </is>
       </c>
       <c r="B9" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Good 2 production and evidence</t>
+          <t xml:space="preserve">Good 2 CN code and evidence</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="5">
@@ -711,12 +711,12 @@
     <row r="10">
       <c r="A10" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">QC_05_1</t>
+          <t xml:space="preserve">QC_04_1</t>
         </is>
       </c>
       <c r="B10" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Good 2 sector</t>
+          <t xml:space="preserve">Good 2 production and evidence</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="5">
@@ -731,19 +731,19 @@
       </c>
       <c r="E10" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">REM_SELECT_SUPPORTED_SECTOR</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">QC_05A</t>
+          <t xml:space="preserve">QC_05_1</t>
         </is>
       </c>
       <c r="B11" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Allocation, evidence and reconciliation</t>
+          <t xml:space="preserve">Good 2 sector</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="5">
@@ -758,19 +758,19 @@
       </c>
       <c r="E11" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">REM_SELECT_SUPPORTED_SECTOR</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">QC_06</t>
+          <t xml:space="preserve">QC_05A</t>
         </is>
       </c>
       <c r="B12" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">directEmissions value, unit and evidence</t>
+          <t xml:space="preserve">Allocation, evidence and reconciliation</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="5">
@@ -792,12 +792,12 @@
     <row r="13">
       <c r="A13" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">QC_07</t>
+          <t xml:space="preserve">QC_06</t>
         </is>
       </c>
       <c r="B13" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">electricityConsumed value, unit and evidence</t>
+          <t xml:space="preserve">directEmissions value, unit and evidence</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="5">
@@ -819,12 +819,12 @@
     <row r="14">
       <c r="A14" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">QC_08</t>
+          <t xml:space="preserve">QC_07</t>
         </is>
       </c>
       <c r="B14" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">gridEmissionFactor value, unit and evidence</t>
+          <t xml:space="preserve">electricityConsumed value, unit and evidence</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="5">
@@ -846,12 +846,12 @@
     <row r="15">
       <c r="A15" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">QC_09</t>
+          <t xml:space="preserve">QC_08</t>
         </is>
       </c>
       <c r="B15" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Precursor scope</t>
+          <t xml:space="preserve">gridEmissionFactor value, unit and evidence</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="5">
@@ -866,19 +866,19 @@
       </c>
       <c r="E15" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">REM_CONFIRM_PRECURSOR_SCOPE</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">QC_10</t>
+          <t xml:space="preserve">QC_09</t>
         </is>
       </c>
       <c r="B16" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Evidence integrity</t>
+          <t xml:space="preserve">Precursor scope</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="5">
@@ -893,39 +893,66 @@
       </c>
       <c r="E16" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">REM_CONFIRM_PRECURSOR_SCOPE</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr" s="1">
         <is>
+          <t xml:space="preserve">QC_10</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Evidence integrity</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr" s="1">
+        <is>
           <t xml:space="preserve">QC_11</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr" s="1">
+      <c r="B18" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Carbon price records</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr" s="1">
+      <c r="C18" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">NOT_APPLICABLE</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr" s="1">
+      <c r="D18" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve"/>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E17"/>
+  <autoFilter ref="A1:E18"/>
   <conditionalFormatting sqref="C2:C1048576">
     <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="PASS">
       <formula>NOT(ISERROR(SEARCH("PASS",C2)))</formula>

</xml_diff>

<commit_message>
fix(readiness): close P0 verifier-trust blockers fail-closed
Stop score renormalization over NOT_ASSESSED weight, block future reporting-period completeness, replace illegal EU 2023/1776 citation with IMPL_2025_2547 SSOT, enforce goods cross-artifact consistency, and drive package component counts from a single contract.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/artifacts/sample-v5/Verifier Workspace.xlsx
+++ b/artifacts/sample-v5/Verifier Workspace.xlsx
@@ -349,7 +349,7 @@
       </c>
       <c r="B8" s="11">
         <f>COUNTIF(QUALITY_CONTROLS!C:C,"PASS")</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C8" t="inlineStr" s="4">
         <is>
@@ -951,8 +951,35 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">QC_12</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Goods cross-artifact consistency</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E18"/>
+  <autoFilter ref="A1:E19"/>
   <conditionalFormatting sqref="C2:C1048576">
     <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="PASS">
       <formula>NOT(ISERROR(SEARCH("PASS",C2)))</formula>

</xml_diff>

<commit_message>
feat(public): ship anonymized field scenarios and SSO cutover explainer
Replace empty case-study slot with sector scenarios, clarify Enterprise SSO IdP/MSA cutover, refresh sample artifacts and sitemap stamps for deploy.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/artifacts/sample-v5/Verifier Workspace.xlsx
+++ b/artifacts/sample-v5/Verifier Workspace.xlsx
@@ -234,12 +234,12 @@
     <row r="3">
       <c r="A3" t="inlineStr" s="4">
         <is>
-          <t xml:space="preserve">Report ID</t>
+          <t xml:space="preserve">Package ID</t>
         </is>
       </c>
       <c r="B3" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">report_aaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaa</t>
+          <t xml:space="preserve">A1111</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="4">
@@ -256,189 +256,211 @@
     <row r="4">
       <c r="A4" t="inlineStr" s="4">
         <is>
+          <t xml:space="preserve">Technical Report ID</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">report_aaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaa</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr" s="4">
+        <is>
           <t xml:space="preserve">Case ID</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr" s="1">
+      <c r="D4" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">case_verifier_grade_fixture</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr" s="4">
-        <is>
-          <t xml:space="preserve">Ruleset</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">3.0.0 · CBAM Definitive Regime 2026</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr" s="4">
         <is>
-          <t xml:space="preserve">Automated readiness</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">READY_FOR_INDEPENDENT_VERIFICATION</t>
+          <t xml:space="preserve">Ruleset</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">3.0.0 · CBAM Definitive Regime 2026</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="4">
         <is>
-          <t xml:space="preserve">Independent verifier status</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">NOT_REVIEWED</t>
+          <t xml:space="preserve">Materiality rate</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">5% per good</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr" s="4">
         <is>
-          <t xml:space="preserve">Calculation root hash</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">7e12ba9592177cc10e0e4541bb103905e0345303fa794949881b86ec2ab48f61</t>
+          <t xml:space="preserve">Automated readiness</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">READY_FOR_INDEPENDENT_VERIFICATION</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="4">
         <is>
-          <t xml:space="preserve">Source registry hash</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">7e17ddb14e300758d5125606820b4ba7e5322c2ee20dd079efe63825990c71bf</t>
+          <t xml:space="preserve">Independent verifier status</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">NOT_REVIEWED</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr" s="4">
         <is>
-          <t xml:space="preserve">Quality controls</t>
+          <t xml:space="preserve">Calculation root hash</t>
         </is>
       </c>
       <c r="B7" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Calculated below</t>
+          <t xml:space="preserve">7e12ba9592177cc10e0e4541bb103905e0345303fa794949881b86ec2ab48f61</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="4">
         <is>
-          <t xml:space="preserve">Materiality rate</t>
+          <t xml:space="preserve">Source registry hash</t>
         </is>
       </c>
       <c r="D7" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">5% per good</t>
+          <t xml:space="preserve">7e17ddb14e300758d5125606820b4ba7e5322c2ee20dd079efe63825990c71bf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr" s="4">
         <is>
+          <t xml:space="preserve">Quality controls</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Calculated below</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Package boundary</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Sealed operator preparation</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr" s="4">
+        <is>
           <t xml:space="preserve">Passed</t>
         </is>
       </c>
-      <c r="B8" s="11">
+      <c r="B9" s="11">
         <f>COUNTIF(QUALITY_CONTROLS!C:C,"PASS")</f>
         <v>16</v>
       </c>
-      <c r="C8" t="inlineStr" s="4">
+      <c r="C9" t="inlineStr" s="4">
         <is>
           <t xml:space="preserve">Blockers</t>
         </is>
       </c>
-      <c r="D8" s="11">
+      <c r="D9" s="11">
         <f>COUNTIF(QUALITY_CONTROLS!C:C,"BLOCKER")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr" s="4">
+    <row r="10">
+      <c r="A10" t="inlineStr" s="4">
         <is>
           <t xml:space="preserve">Warnings</t>
         </is>
       </c>
-      <c r="B9" s="11">
+      <c r="B10" s="11">
         <f>COUNTIF(QUALITY_CONTROLS!C:C,"WARNING")</f>
         <v>0</v>
       </c>
-      <c r="C9" t="inlineStr" s="4">
+      <c r="C10" t="inlineStr" s="4">
         <is>
           <t xml:space="preserve">Monitoring-plan gaps</t>
         </is>
       </c>
-      <c r="D9" s="11">
+      <c r="D10" s="11">
         <f>COUNTIF(MONITORING_PLAN!C:C,"GAP")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr" s="4">
+    <row r="11">
+      <c r="A11" t="inlineStr" s="4">
         <is>
           <t xml:space="preserve">Evidence files</t>
         </is>
       </c>
-      <c r="B10" s="11">
+      <c r="B11" s="11">
         <f>COUNTA(EVIDENCE!A2:A1048576)</f>
         <v>4</v>
       </c>
-      <c r="C10" t="inlineStr" s="4">
+      <c r="C11" t="inlineStr" s="4">
         <is>
           <t xml:space="preserve">Approved clean evidence</t>
         </is>
       </c>
-      <c r="D10" s="8">
+      <c r="D11" s="8">
         <v>4</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr" s="4">
-        <is>
-          <t xml:space="preserve">Evidence coverage</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">100%</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr" s="4">
-        <is>
-          <t xml:space="preserve">Duplicate hashes</t>
-        </is>
-      </c>
-      <c r="D11" s="5">
-        <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr" s="4">
         <is>
-          <t xml:space="preserve">Package boundary</t>
+          <t xml:space="preserve">Evidence coverage</t>
         </is>
       </c>
       <c r="B12" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">This package supports preparation for independent verification. It is not a verification opinion, accreditation decision, customs decision, CBAM Registry submission or acceptance guarantee.</t>
-        </is>
+          <t xml:space="preserve">100%</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Duplicate hashes</t>
+        </is>
+      </c>
+      <c r="D12" s="5">
+        <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr" s="4">
         <is>
+          <t xml:space="preserve">Package boundary</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">This package supports preparation for independent verification. It is not a verification opinion, accreditation decision, customs decision, CBAM Registry submission or acceptance guarantee.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr" s="4">
+        <is>
           <t xml:space="preserve">Instructions</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr" s="1">
+      <c r="B14" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Review QUALITY_CONTROLS, MONITORING_PLAN, EVIDENCE, METHODS and CALCULATION_TRACE. Record independent conclusions only in VERIFIER_SIGN_OFF. Do not overwrite sealed source data.</t>
         </is>

</xml_diff>

<commit_message>
fix(dossier): Annex II priced SEE, origin hard-block, honest evidence/crypto claims
Root-cause remediation for S0176-class defects: sector rules exclude indirect from CBAM-priced SEE for Annex II goods; EU/Annex III origins hard-block sealing; evidence MIME/concentration rules stop one-file 100% scores; KMS FIPS claims derive from protectionLevel; offline verify CLI ships in packages; SEO docs regenerated.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/artifacts/sample-v5/Verifier Workspace.xlsx
+++ b/artifacts/sample-v5/Verifier Workspace.xlsx
@@ -327,7 +327,7 @@
       </c>
       <c r="B7" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">7e12ba9592177cc10e0e4541bb103905e0345303fa794949881b86ec2ab48f61</t>
+          <t xml:space="preserve">179d2547250f42d58eb1b1a3c79283294ad74c4f4568871a6ff6fed5d94f5418</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="4">
@@ -371,7 +371,7 @@
       </c>
       <c r="B9" s="11">
         <f>COUNTIF(QUALITY_CONTROLS!C:C,"PASS")</f>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C9" t="inlineStr" s="4">
         <is>
@@ -571,12 +571,12 @@
     <row r="4">
       <c r="A4" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">QC_01</t>
+          <t xml:space="preserve">QC_00_ORIGIN</t>
         </is>
       </c>
       <c r="B4" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">EORI format and evidence</t>
+          <t xml:space="preserve">Installation country of origin CBAM scope</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="5">
@@ -598,12 +598,12 @@
     <row r="5">
       <c r="A5" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">QC_02</t>
+          <t xml:space="preserve">QC_01</t>
         </is>
       </c>
       <c r="B5" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Definitive-period reporting year</t>
+          <t xml:space="preserve">EORI format and evidence</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="5">
@@ -618,19 +618,19 @@
       </c>
       <c r="E5" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">REM_CORRECT_REPORTING_YEAR</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">QC_03_0</t>
+          <t xml:space="preserve">QC_02</t>
         </is>
       </c>
       <c r="B6" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Good 1 CN code and evidence</t>
+          <t xml:space="preserve">Definitive-period reporting year</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="5">
@@ -645,19 +645,19 @@
       </c>
       <c r="E6" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">REM_CORRECT_REPORTING_YEAR</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">QC_04_0</t>
+          <t xml:space="preserve">QC_03_0</t>
         </is>
       </c>
       <c r="B7" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Good 1 production and evidence</t>
+          <t xml:space="preserve">Good 1 CN code and evidence</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="5">
@@ -679,12 +679,12 @@
     <row r="8">
       <c r="A8" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">QC_05_0</t>
+          <t xml:space="preserve">QC_04_0</t>
         </is>
       </c>
       <c r="B8" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Good 1 sector</t>
+          <t xml:space="preserve">Good 1 production and evidence</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="5">
@@ -699,19 +699,19 @@
       </c>
       <c r="E8" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">REM_SELECT_SUPPORTED_SECTOR</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">QC_03_1</t>
+          <t xml:space="preserve">QC_05_0</t>
         </is>
       </c>
       <c r="B9" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Good 2 CN code and evidence</t>
+          <t xml:space="preserve">Good 1 sector</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="5">
@@ -726,19 +726,19 @@
       </c>
       <c r="E9" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">REM_SELECT_SUPPORTED_SECTOR</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">QC_04_1</t>
+          <t xml:space="preserve">QC_03_1</t>
         </is>
       </c>
       <c r="B10" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Good 2 production and evidence</t>
+          <t xml:space="preserve">Good 2 CN code and evidence</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="5">
@@ -760,12 +760,12 @@
     <row r="11">
       <c r="A11" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">QC_05_1</t>
+          <t xml:space="preserve">QC_04_1</t>
         </is>
       </c>
       <c r="B11" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Good 2 sector</t>
+          <t xml:space="preserve">Good 2 production and evidence</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="5">
@@ -780,19 +780,19 @@
       </c>
       <c r="E11" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">REM_SELECT_SUPPORTED_SECTOR</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">QC_05A</t>
+          <t xml:space="preserve">QC_05_1</t>
         </is>
       </c>
       <c r="B12" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Allocation, evidence and reconciliation</t>
+          <t xml:space="preserve">Good 2 sector</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="5">
@@ -807,19 +807,19 @@
       </c>
       <c r="E12" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">REM_SELECT_SUPPORTED_SECTOR</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">QC_06</t>
+          <t xml:space="preserve">QC_05A</t>
         </is>
       </c>
       <c r="B13" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">directEmissions value, unit and evidence</t>
+          <t xml:space="preserve">Allocation, evidence and reconciliation</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="5">
@@ -841,12 +841,12 @@
     <row r="14">
       <c r="A14" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">QC_07</t>
+          <t xml:space="preserve">QC_06</t>
         </is>
       </c>
       <c r="B14" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">electricityConsumed value, unit and evidence</t>
+          <t xml:space="preserve">directEmissions value, unit and evidence</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="5">
@@ -868,12 +868,12 @@
     <row r="15">
       <c r="A15" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">QC_08</t>
+          <t xml:space="preserve">QC_07</t>
         </is>
       </c>
       <c r="B15" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">gridEmissionFactor value, unit and evidence</t>
+          <t xml:space="preserve">electricityConsumed value, unit and evidence</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="5">
@@ -895,12 +895,12 @@
     <row r="16">
       <c r="A16" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">QC_09</t>
+          <t xml:space="preserve">QC_08</t>
         </is>
       </c>
       <c r="B16" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Precursor scope</t>
+          <t xml:space="preserve">gridEmissionFactor value, unit and evidence</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="5">
@@ -915,19 +915,19 @@
       </c>
       <c r="E16" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">REM_CONFIRM_PRECURSOR_SCOPE</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">QC_10</t>
+          <t xml:space="preserve">QC_09</t>
         </is>
       </c>
       <c r="B17" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Evidence integrity</t>
+          <t xml:space="preserve">Precursor scope</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="5">
@@ -942,24 +942,24 @@
       </c>
       <c r="E17" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">REM_CONFIRM_PRECURSOR_SCOPE</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">QC_11</t>
+          <t xml:space="preserve">QC_10</t>
         </is>
       </c>
       <c r="B18" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Carbon price records</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">NOT_APPLICABLE</t>
+          <t xml:space="preserve">Evidence integrity</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">PASS</t>
         </is>
       </c>
       <c r="D18" t="inlineStr" s="1">
@@ -976,32 +976,59 @@
     <row r="19">
       <c r="A19" t="inlineStr" s="1">
         <is>
+          <t xml:space="preserve">QC_11</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Carbon price records</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">NOT_APPLICABLE</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr" s="1">
+        <is>
           <t xml:space="preserve">QC_12</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr" s="1">
+      <c r="B20" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Goods cross-artifact consistency</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr" s="5">
+      <c r="C20" t="inlineStr" s="5">
         <is>
           <t xml:space="preserve">PASS</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr" s="1">
+      <c r="D20" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve"/>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E19"/>
+  <autoFilter ref="A1:E20"/>
   <conditionalFormatting sqref="C2:C1048576">
     <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="PASS">
       <formula>NOT(ISERROR(SEARCH("PASS",C2)))</formula>
@@ -1075,17 +1102,17 @@
     <row r="2">
       <c r="A2" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">calc_445d0057447929d658bf459d98dc777e</t>
+          <t xml:space="preserve">calc_7e1498210522444ae03dbb6106b3a5cb</t>
         </is>
       </c>
       <c r="B2" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">CBAM_INDIRECT_EMISSIONS</t>
+          <t xml:space="preserve">CBAM_INSTALLATION_DIRECT_EMISSIONS</t>
         </is>
       </c>
       <c r="C2" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">40</t>
+          <t xml:space="preserve">80</t>
         </is>
       </c>
       <c r="D2" t="inlineStr" s="1">
@@ -1095,7 +1122,7 @@
       </c>
       <c r="E2" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">6a2647d365280b1a97c749006dfaa066e9374f7534b8c11cafe32b791c010350</t>
+          <t xml:space="preserve">690085cd04f6102b1d2617fa92b671e089632e2db84f8c657a521938be42eb57</t>
         </is>
       </c>
       <c r="F2" t="inlineStr" s="1">
@@ -1107,17 +1134,17 @@
     <row r="3">
       <c r="A3" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">calc_1630e8db831bb1cb37c6a7198e0ae9c5</t>
+          <t xml:space="preserve">calc_90bff6dba51677ea832d6a39caa9cb59</t>
         </is>
       </c>
       <c r="B3" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">CBAM_PRECURSOR_EMISSIONS_SUM</t>
+          <t xml:space="preserve">CBAM_INDIRECT_EMISSIONS</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">0</t>
+          <t xml:space="preserve">40</t>
         </is>
       </c>
       <c r="D3" t="inlineStr" s="1">
@@ -1127,7 +1154,7 @@
       </c>
       <c r="E3" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">5553fb3ff7a2d2d3f04af35bdcb6f4c64f77ee3359321812bc30163f210d3c86</t>
+          <t xml:space="preserve">98a76aac49f58cbd4c0ad68637e03e592b2dd2e0bc7208a8062648de29ffe081</t>
         </is>
       </c>
       <c r="F3" t="inlineStr" s="1">
@@ -1139,17 +1166,17 @@
     <row r="4">
       <c r="A4" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">calc_f13dfcef59790232c64b830522fbab3e</t>
+          <t xml:space="preserve">calc_1630e8db831bb1cb37c6a7198e0ae9c5</t>
         </is>
       </c>
       <c r="B4" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">CBAM_TOTAL_EMBEDDED_EMISSIONS</t>
+          <t xml:space="preserve">CBAM_PRECURSOR_EMISSIONS_SUM</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">120</t>
+          <t xml:space="preserve">0</t>
         </is>
       </c>
       <c r="D4" t="inlineStr" s="1">
@@ -1159,7 +1186,7 @@
       </c>
       <c r="E4" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">cc192e8f6a78218e061c33a7c0a99f82059fba5ee1def6dd1735ccabc099b2d2</t>
+          <t xml:space="preserve">5553fb3ff7a2d2d3f04af35bdcb6f4c64f77ee3359321812bc30163f210d3c86</t>
         </is>
       </c>
       <c r="F4" t="inlineStr" s="1">
@@ -1171,49 +1198,49 @@
     <row r="5">
       <c r="A5" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">calc_392b30d9018c8523ee80c07eca731011</t>
+          <t xml:space="preserve">calc_51d89a66ef242ddb996ab391a4bc0675</t>
         </is>
       </c>
       <c r="B5" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">CBAM_GOOD_EMISSIONS_ALLOCATION_1</t>
+          <t xml:space="preserve">CBAM_TOTAL_EMBEDDED_EMISSIONS_DISCLOSED</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">1.2</t>
+          <t xml:space="preserve">120</t>
         </is>
       </c>
       <c r="D5" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">tCO2e/t</t>
+          <t xml:space="preserve">tCO2e</t>
         </is>
       </c>
       <c r="E5" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">7aba824be81004f963dadb979458428808b42ab7d4f48dbfcae56a4f661fd5ba</t>
+          <t xml:space="preserve">3bd0d06237ae6b808a635fb731efb40b74fb90a51e42bfe49ed064cb41f03e2f</t>
         </is>
       </c>
       <c r="F5" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Disclosed total combines direct and indirect emissions before sector-specific pricing rules.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">calc_a7674a302f1435ec031cc0aece62e1fe</t>
+          <t xml:space="preserve">calc_c9b675a88bbe12e9e0499e2c41146bd4</t>
         </is>
       </c>
       <c r="B6" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">CBAM_GOOD_EMISSIONS_ALLOCATION_2</t>
+          <t xml:space="preserve">CBAM_GOOD_EMISSIONS_ALLOCATION_1</t>
         </is>
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">1.2</t>
+          <t xml:space="preserve">0.8</t>
         </is>
       </c>
       <c r="D6" t="inlineStr" s="1">
@@ -1223,7 +1250,7 @@
       </c>
       <c r="E6" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">2d6d72ee83e4cd16157fe19d8f21971c0c6b8e36076c5bbbf42403b5a39f5a9b</t>
+          <t xml:space="preserve">137fc83c1e53a213bd38caccb4359607638050549305b90e340da30d856a26c1</t>
         </is>
       </c>
       <c r="F6" t="inlineStr" s="1">
@@ -1235,27 +1262,27 @@
     <row r="7">
       <c r="A7" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">calc_73dbfc45799a70fdbc9a491dc6506d4e</t>
+          <t xml:space="preserve">calc_abc058b793bf631c47e250d0e59d3959</t>
         </is>
       </c>
       <c r="B7" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">CBAM_GOODS_ALLOCATION_RECONCILIATION</t>
+          <t xml:space="preserve">CBAM_GOOD_EMISSIONS_ALLOCATION_2</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">0</t>
+          <t xml:space="preserve">0.8</t>
         </is>
       </c>
       <c r="D7" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">tCO2e</t>
+          <t xml:space="preserve">tCO2e/t</t>
         </is>
       </c>
       <c r="E7" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">274077c9bd67745642e0aaf8506b146e80db2fca464cbcbf55485d95475c2fd0</t>
+          <t xml:space="preserve">2670d4a69b964809495520ced63320b6cced57f17d354d9a422aaf1b7c7df0e9</t>
         </is>
       </c>
       <c r="F7" t="inlineStr" s="1">
@@ -1267,69 +1294,133 @@
     <row r="8">
       <c r="A8" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">calc_b1cd714bbd7ee6e74fcc264bb2ced3ba</t>
+          <t xml:space="preserve">calc_fd4f5ff4cf9362acbac25669641f9d5c</t>
         </is>
       </c>
       <c r="B8" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">CBAM_AGGREGATE_SPECIFIC_EMBEDDED_EMISSIONS</t>
+          <t xml:space="preserve">CBAM_TOTAL_EMBEDDED_EMISSIONS_PRICED</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">1.2</t>
+          <t xml:space="preserve">80</t>
         </is>
       </c>
       <c r="D8" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">tCO2e/t</t>
+          <t xml:space="preserve">tCO2e</t>
         </is>
       </c>
       <c r="E8" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">61fff4226612cedc54b2fdf528abe1b84fd63436a2cef5e27dc6b2f41761f2d0</t>
+          <t xml:space="preserve">1b547bb68197cb8f0357a93b9cd6f8655d4cac8c062d1840050938f4a7d82966</t>
         </is>
       </c>
       <c r="F8" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">The aggregate intensity is a portfolio diagnostic; reportable values are the per-good intensities.</t>
+          <t xml:space="preserve">Priced total applies sector Annex II direct-only rules where applicable.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr" s="1">
         <is>
+          <t xml:space="preserve">calc_b59727b834166a6e86a4fb168d149e1d</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">CBAM_GOODS_ALLOCATION_RECONCILIATION</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">0</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">tCO2e</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">a507c7fe68ea6bff1451969dc6b94557b316689ea670e3948498cd1d3750091b</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">calc_d6b26df091b143960b5c2beae3f6324e</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">CBAM_AGGREGATE_SPECIFIC_EMBEDDED_EMISSIONS</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">0.8</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">tCO2e/t</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">ead9fddcade625553ba96d6a41e1913ed8e8ad1c03b6cf1b955e59c5272b795e</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">The aggregate intensity is a portfolio diagnostic; reportable values are the per-good intensities.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr" s="1">
+        <is>
           <t xml:space="preserve">calc_bc235e307191b831ced1965ffd282183</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr" s="1">
+      <c r="B11" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">CBAM_CARBON_PRICE_REDUCTION_RECORD_TOTAL</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr" s="1">
+      <c r="C11" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">0</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr" s="1">
+      <c r="D11" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">certificate-equivalent</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr" s="1">
+      <c r="E11" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">13eee823710e59782162be2fd529ca7dd9bb3ac7b195d5d21486017266c848ea</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr" s="1">
+      <c r="F11" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve"/>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F9"/>
+  <autoFilter ref="A1:F11"/>
   <printOptions horizontalCentered="0" verticalCentered="0"/>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0" paperSize="9"/>
@@ -2044,7 +2135,7 @@
       </c>
       <c r="B5" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Verified Steel Operator GmbH</t>
+          <t xml:space="preserve">Verified Steel Operator A.S.</t>
         </is>
       </c>
       <c r="C5" t="inlineStr" s="1">
@@ -2088,7 +2179,7 @@
       </c>
       <c r="B7" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">DE</t>
+          <t xml:space="preserve">TR</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="1">
@@ -2296,20 +2387,20 @@
         <v>0.6</v>
       </c>
       <c r="G2" s="8">
-        <v>72</v>
+        <v>48</v>
       </c>
       <c r="H2" s="8">
-        <v>1.2</v>
+        <v>0.8</v>
       </c>
       <c r="I2" s="8">
         <v>5</v>
       </c>
       <c r="J2" s="8">
-        <v>0.06</v>
+        <v>0.04</v>
       </c>
       <c r="K2" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">calc_392b30d9018c8523ee80c07eca731011</t>
+          <t xml:space="preserve">calc_c9b675a88bbe12e9e0499e2c41146bd4</t>
         </is>
       </c>
     </row>
@@ -2339,20 +2430,20 @@
         <v>0.4</v>
       </c>
       <c r="G3" s="8">
-        <v>48</v>
+        <v>32</v>
       </c>
       <c r="H3" s="8">
-        <v>1.2</v>
+        <v>0.8</v>
       </c>
       <c r="I3" s="8">
         <v>5</v>
       </c>
       <c r="J3" s="8">
-        <v>0.06</v>
+        <v>0.04</v>
       </c>
       <c r="K3" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">calc_a7674a302f1435ec031cc0aece62e1fe</t>
+          <t xml:space="preserve">calc_abc058b793bf631c47e250d0e59d3959</t>
         </is>
       </c>
     </row>
@@ -2526,7 +2617,7 @@
         </is>
       </c>
       <c r="B8" s="8">
-        <v>120</v>
+        <v>80</v>
       </c>
       <c r="C8" t="inlineStr" s="1">
         <is>
@@ -2566,7 +2657,7 @@
         </is>
       </c>
       <c r="B10" s="8">
-        <v>1.2</v>
+        <v>0.8</v>
       </c>
       <c r="C10" t="inlineStr" s="1">
         <is>
@@ -2976,7 +3067,7 @@
       </c>
       <c r="C2" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">customs-declaration-classification.txt</t>
+          <t xml:space="preserve">customs-declaration-classification.pdf</t>
         </is>
       </c>
       <c r="D2" t="inlineStr" s="1">
@@ -3031,7 +3122,7 @@
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">electricity-utility-invoice.txt</t>
+          <t xml:space="preserve">electricity-utility-invoice.pdf</t>
         </is>
       </c>
       <c r="D3" t="inlineStr" s="1">
@@ -3086,7 +3177,7 @@
       </c>
       <c r="C4" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">production-reconciliation-ledger.txt</t>
+          <t xml:space="preserve">production-reconciliation-ledger.pdf</t>
         </is>
       </c>
       <c r="D4" t="inlineStr" s="1">
@@ -3141,7 +3232,7 @@
       </c>
       <c r="C5" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">verified-monitoring-package.txt</t>
+          <t xml:space="preserve">verified-monitoring-package.pdf</t>
         </is>
       </c>
       <c r="D5" t="inlineStr" s="1">
@@ -3561,7 +3652,7 @@
       </c>
       <c r="D8" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">8 hashed trace node(s)</t>
+          <t xml:space="preserve">10 hashed trace node(s)</t>
         </is>
       </c>
     </row>
@@ -3671,7 +3762,7 @@
       </c>
       <c r="D13" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Calculation root 7e12ba9592177cc10e0e4541bb103905e0345303fa794949881b86ec2ab48f61</t>
+          <t xml:space="preserve">Calculation root 179d2547250f42d58eb1b1a3c79283294ad74c4f4568871a6ff6fed5d94f5418</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(dossier): wizard guidance, structured evidence quality, four complete sandbox dossiers (#82)
Final P0 release patch for mandatory-field wizard guidance, structured evidence grading, methodology-decision controls, and four complete sandbox dossiers.
</commit_message>
<xml_diff>
--- a/artifacts/sample-v5/Verifier Workspace.xlsx
+++ b/artifacts/sample-v5/Verifier Workspace.xlsx
@@ -4306,7 +4306,7 @@
       </c>
       <c r="E2" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Evidence check failed with status 'PARTIALLY_SUPPORTED'. Reason codes: SINGLE_SOURCE_CONCENTRATION, EVIDENCE_DIVERSITY_INSUFFICIENT</t>
+          <t xml:space="preserve">Evidence check failed with status 'PARTIALLY_SUPPORTED'. Reason codes: MATERIAL_EVIDENCE_QUALITY_D_OR_E, SINGLE_SOURCE_CONCENTRATION, EVIDENCE_DIVERSITY_INSUFFICIENT</t>
         </is>
       </c>
       <c r="F2" t="inlineStr" s="1">
@@ -4338,7 +4338,7 @@
       </c>
       <c r="E3" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Evidence check failed with status 'PARTIALLY_SUPPORTED'. Reason codes: SINGLE_SOURCE_CONCENTRATION, EVIDENCE_DIVERSITY_INSUFFICIENT</t>
+          <t xml:space="preserve">Evidence check failed with status 'PARTIALLY_SUPPORTED'. Reason codes: MATERIAL_EVIDENCE_QUALITY_D_OR_E, SINGLE_SOURCE_CONCENTRATION, EVIDENCE_DIVERSITY_INSUFFICIENT</t>
         </is>
       </c>
       <c r="F3" t="inlineStr" s="1">
@@ -4370,7 +4370,7 @@
       </c>
       <c r="E4" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Evidence check failed with status 'PARTIALLY_SUPPORTED'. Reason codes: SINGLE_SOURCE_CONCENTRATION, EVIDENCE_DIVERSITY_INSUFFICIENT</t>
+          <t xml:space="preserve">Evidence check failed with status 'PARTIALLY_SUPPORTED'. Reason codes: MATERIAL_EVIDENCE_QUALITY_D_OR_E, SINGLE_SOURCE_CONCENTRATION, EVIDENCE_DIVERSITY_INSUFFICIENT</t>
         </is>
       </c>
       <c r="F4" t="inlineStr" s="1">
@@ -4402,7 +4402,7 @@
       </c>
       <c r="E5" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Evidence check failed with status 'PARTIALLY_SUPPORTED'. Reason codes: SINGLE_SOURCE_CONCENTRATION, EVIDENCE_DIVERSITY_INSUFFICIENT</t>
+          <t xml:space="preserve">Evidence check failed with status 'PARTIALLY_SUPPORTED'. Reason codes: MATERIAL_EVIDENCE_QUALITY_D_OR_E, SINGLE_SOURCE_CONCENTRATION, EVIDENCE_DIVERSITY_INSUFFICIENT</t>
         </is>
       </c>
       <c r="F5" t="inlineStr" s="1">
@@ -4434,7 +4434,7 @@
       </c>
       <c r="E6" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Evidence check failed with status 'PARTIALLY_SUPPORTED'. Reason codes: SINGLE_SOURCE_CONCENTRATION, EVIDENCE_DIVERSITY_INSUFFICIENT</t>
+          <t xml:space="preserve">Evidence check failed with status 'PARTIALLY_SUPPORTED'. Reason codes: MATERIAL_EVIDENCE_QUALITY_D_OR_E, SINGLE_SOURCE_CONCENTRATION, EVIDENCE_DIVERSITY_INSUFFICIENT</t>
         </is>
       </c>
       <c r="F6" t="inlineStr" s="1">
@@ -4466,7 +4466,7 @@
       </c>
       <c r="E7" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Evidence check failed with status 'PARTIALLY_SUPPORTED'. Reason codes: SINGLE_SOURCE_CONCENTRATION, EVIDENCE_DIVERSITY_INSUFFICIENT</t>
+          <t xml:space="preserve">Evidence check failed with status 'PARTIALLY_SUPPORTED'. Reason codes: MATERIAL_EVIDENCE_QUALITY_D_OR_E, SINGLE_SOURCE_CONCENTRATION, EVIDENCE_DIVERSITY_INSUFFICIENT</t>
         </is>
       </c>
       <c r="F7" t="inlineStr" s="1">
@@ -4498,7 +4498,7 @@
       </c>
       <c r="E8" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Evidence check failed with status 'PARTIALLY_SUPPORTED'. Reason codes: SINGLE_SOURCE_CONCENTRATION, EVIDENCE_DIVERSITY_INSUFFICIENT</t>
+          <t xml:space="preserve">Evidence check failed with status 'PARTIALLY_SUPPORTED'. Reason codes: MATERIAL_EVIDENCE_QUALITY_D_OR_E, SINGLE_SOURCE_CONCENTRATION, EVIDENCE_DIVERSITY_INSUFFICIENT</t>
         </is>
       </c>
       <c r="F8" t="inlineStr" s="1">
@@ -4562,7 +4562,7 @@
       </c>
       <c r="E10" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Evidence check failed with status 'PARTIALLY_SUPPORTED'. Reason codes: SINGLE_SOURCE_CONCENTRATION, EVIDENCE_DIVERSITY_INSUFFICIENT</t>
+          <t xml:space="preserve">Evidence check failed with status 'PARTIALLY_SUPPORTED'. Reason codes: MATERIAL_EVIDENCE_QUALITY_D_OR_E, SINGLE_SOURCE_CONCENTRATION, EVIDENCE_DIVERSITY_INSUFFICIENT</t>
         </is>
       </c>
       <c r="F10" t="inlineStr" s="1">
@@ -4594,7 +4594,7 @@
       </c>
       <c r="E11" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Evidence check failed with status 'PARTIALLY_SUPPORTED'. Reason codes: SINGLE_SOURCE_CONCENTRATION, EVIDENCE_DIVERSITY_INSUFFICIENT</t>
+          <t xml:space="preserve">Evidence check failed with status 'PARTIALLY_SUPPORTED'. Reason codes: MATERIAL_EVIDENCE_QUALITY_D_OR_E, SINGLE_SOURCE_CONCENTRATION, EVIDENCE_DIVERSITY_INSUFFICIENT</t>
         </is>
       </c>
       <c r="F11" t="inlineStr" s="1">
@@ -4626,7 +4626,7 @@
       </c>
       <c r="E12" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Evidence check failed with status 'PARTIALLY_SUPPORTED'. Reason codes: EVIDENCE_DIVERSITY_INSUFFICIENT</t>
+          <t xml:space="preserve">Evidence check failed with status 'PARTIALLY_SUPPORTED'. Reason codes: MATERIAL_EVIDENCE_QUALITY_D_OR_E, EVIDENCE_DIVERSITY_INSUFFICIENT</t>
         </is>
       </c>
       <c r="F12" t="inlineStr" s="1">
@@ -4690,7 +4690,7 @@
       </c>
       <c r="E14" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Evidence check failed with status 'PARTIALLY_SUPPORTED'. Reason codes: SINGLE_SOURCE_CONCENTRATION, EVIDENCE_DIVERSITY_INSUFFICIENT</t>
+          <t xml:space="preserve">Evidence check failed with status 'PARTIALLY_SUPPORTED'. Reason codes: MATERIAL_EVIDENCE_QUALITY_D_OR_E, SINGLE_SOURCE_CONCENTRATION, EVIDENCE_DIVERSITY_INSUFFICIENT</t>
         </is>
       </c>
       <c r="F14" t="inlineStr" s="1">
@@ -4722,7 +4722,7 @@
       </c>
       <c r="E15" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Evidence check failed with status 'PARTIALLY_SUPPORTED'. Reason codes: EVIDENCE_DIVERSITY_INSUFFICIENT</t>
+          <t xml:space="preserve">Evidence check failed with status 'PARTIALLY_SUPPORTED'. Reason codes: MATERIAL_EVIDENCE_QUALITY_D_OR_E, EVIDENCE_DIVERSITY_INSUFFICIENT</t>
         </is>
       </c>
       <c r="F15" t="inlineStr" s="1">
@@ -4786,7 +4786,7 @@
       </c>
       <c r="E17" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Evidence check failed with status 'PARTIALLY_SUPPORTED'. Reason codes: EVIDENCE_DIVERSITY_INSUFFICIENT</t>
+          <t xml:space="preserve">Evidence check failed with status 'PARTIALLY_SUPPORTED'. Reason codes: MATERIAL_EVIDENCE_QUALITY_D_OR_E, EVIDENCE_DIVERSITY_INSUFFICIENT</t>
         </is>
       </c>
       <c r="F17" t="inlineStr" s="1">
@@ -4818,7 +4818,7 @@
       </c>
       <c r="E18" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Evidence check failed with status 'PARTIALLY_SUPPORTED'. Reason codes: EVIDENCE_DIVERSITY_INSUFFICIENT</t>
+          <t xml:space="preserve">Evidence check failed with status 'PARTIALLY_SUPPORTED'. Reason codes: MATERIAL_EVIDENCE_QUALITY_D_OR_E, EVIDENCE_DIVERSITY_INSUFFICIENT</t>
         </is>
       </c>
       <c r="F18" t="inlineStr" s="1">
@@ -4850,7 +4850,7 @@
       </c>
       <c r="E19" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Evidence check failed with status 'PARTIALLY_SUPPORTED'. Reason codes: EVIDENCE_DIVERSITY_INSUFFICIENT</t>
+          <t xml:space="preserve">Evidence check failed with status 'PARTIALLY_SUPPORTED'. Reason codes: MATERIAL_EVIDENCE_QUALITY_D_OR_E, EVIDENCE_DIVERSITY_INSUFFICIENT</t>
         </is>
       </c>
       <c r="F19" t="inlineStr" s="1">
@@ -6466,7 +6466,7 @@
       </c>
       <c r="I2" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">SINGLE_SOURCE_CONCENTRATION | EVIDENCE_DIVERSITY_INSUFFICIENT</t>
+          <t xml:space="preserve">MATERIAL_EVIDENCE_QUALITY_D_OR_E | SINGLE_SOURCE_CONCENTRATION | EVIDENCE_DIVERSITY_INSUFFICIENT</t>
         </is>
       </c>
     </row>
@@ -6701,7 +6701,7 @@
       </c>
       <c r="I7" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">SINGLE_SOURCE_CONCENTRATION | EVIDENCE_DIVERSITY_INSUFFICIENT</t>
+          <t xml:space="preserve">MATERIAL_EVIDENCE_QUALITY_D_OR_E | SINGLE_SOURCE_CONCENTRATION | EVIDENCE_DIVERSITY_INSUFFICIENT</t>
         </is>
       </c>
     </row>
@@ -7359,7 +7359,7 @@
       </c>
       <c r="I21" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">SINGLE_SOURCE_CONCENTRATION | EVIDENCE_DIVERSITY_INSUFFICIENT</t>
+          <t xml:space="preserve">MATERIAL_EVIDENCE_QUALITY_D_OR_E | SINGLE_SOURCE_CONCENTRATION | EVIDENCE_DIVERSITY_INSUFFICIENT</t>
         </is>
       </c>
     </row>
@@ -7406,7 +7406,7 @@
       </c>
       <c r="I22" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">EVIDENCE_DIVERSITY_INSUFFICIENT</t>
+          <t xml:space="preserve">MATERIAL_EVIDENCE_QUALITY_D_OR_E | EVIDENCE_DIVERSITY_INSUFFICIENT</t>
         </is>
       </c>
     </row>
@@ -7500,7 +7500,7 @@
       </c>
       <c r="I24" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">SINGLE_SOURCE_CONCENTRATION | EVIDENCE_DIVERSITY_INSUFFICIENT</t>
+          <t xml:space="preserve">MATERIAL_EVIDENCE_QUALITY_D_OR_E | SINGLE_SOURCE_CONCENTRATION | EVIDENCE_DIVERSITY_INSUFFICIENT</t>
         </is>
       </c>
     </row>
@@ -7547,7 +7547,7 @@
       </c>
       <c r="I25" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">EVIDENCE_DIVERSITY_INSUFFICIENT</t>
+          <t xml:space="preserve">MATERIAL_EVIDENCE_QUALITY_D_OR_E | EVIDENCE_DIVERSITY_INSUFFICIENT</t>
         </is>
       </c>
     </row>
@@ -7641,7 +7641,7 @@
       </c>
       <c r="I27" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">EVIDENCE_DIVERSITY_INSUFFICIENT</t>
+          <t xml:space="preserve">MATERIAL_EVIDENCE_QUALITY_D_OR_E | EVIDENCE_DIVERSITY_INSUFFICIENT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(wizard): unify guided workflow and prove four sandbox dossiers
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/artifacts/sample-v5/Verifier Workspace.xlsx
+++ b/artifacts/sample-v5/Verifier Workspace.xlsx
@@ -391,7 +391,7 @@
       </c>
       <c r="B9" s="11">
         <f>COUNTIF(QUALITY_CONTROLS!C:C,"PASS")</f>
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C9" t="inlineStr" s="4">
         <is>
@@ -997,32 +997,59 @@
     <row r="19">
       <c r="A19" t="inlineStr" s="1">
         <is>
+          <t xml:space="preserve">QC_11_55555555-5555-4555-8555-555555555555</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Carbon price proof</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr" s="1">
+        <is>
           <t xml:space="preserve">QC_12</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr" s="1">
+      <c r="B20" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Goods cross-artifact consistency</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr" s="5">
+      <c r="C20" t="inlineStr" s="5">
         <is>
           <t xml:space="preserve">PASS</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr" s="1">
+      <c r="D20" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve"/>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E19"/>
+  <autoFilter ref="A1:E20"/>
   <sheetProtection sheet="1" objects="1" scenarios="1" selectLockedCells="1" selectUnlockedCells="1" formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
   <conditionalFormatting sqref="C2:C1048576">
     <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="PASS">

</xml_diff>

<commit_message>
fix(wizard): unify guided workflow and prove four sandbox dossiers (#88)
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/artifacts/sample-v5/Verifier Workspace.xlsx
+++ b/artifacts/sample-v5/Verifier Workspace.xlsx
@@ -391,7 +391,7 @@
       </c>
       <c r="B9" s="11">
         <f>COUNTIF(QUALITY_CONTROLS!C:C,"PASS")</f>
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C9" t="inlineStr" s="4">
         <is>
@@ -997,32 +997,59 @@
     <row r="19">
       <c r="A19" t="inlineStr" s="1">
         <is>
+          <t xml:space="preserve">QC_11_55555555-5555-4555-8555-555555555555</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Carbon price proof</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">PASS</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr" s="1">
+        <is>
           <t xml:space="preserve">QC_12</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr" s="1">
+      <c r="B20" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">Goods cross-artifact consistency</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr" s="5">
+      <c r="C20" t="inlineStr" s="5">
         <is>
           <t xml:space="preserve">PASS</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr" s="1">
+      <c r="D20" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve"/>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E19"/>
+  <autoFilter ref="A1:E20"/>
   <sheetProtection sheet="1" objects="1" scenarios="1" selectLockedCells="1" selectUnlockedCells="1" formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
   <conditionalFormatting sqref="C2:C1048576">
     <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="PASS">

</xml_diff>

<commit_message>
fix(step8): add premium release command center
</commit_message>
<xml_diff>
--- a/artifacts/sample-v5/Verifier Workspace.xlsx
+++ b/artifacts/sample-v5/Verifier Workspace.xlsx
@@ -4245,12 +4245,12 @@
       </c>
       <c r="E2" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">The reporting period end date is in the future relative to the assessment timestamp. Future periods are blocked from sealing.</t>
+          <t xml:space="preserve">The structurally complete annual reporting period ends in the future. A conditional operator working file may be generated, but definitive annual readiness and verifier handover remain blocked.</t>
         </is>
       </c>
       <c r="F2" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Invalid, future, or incomplete reporting period dates block sealing and readiness.</t>
+          <t xml:space="preserve">A future annual period blocks definitive readiness and verifier handover, but not an explicitly conditional operator working file.</t>
         </is>
       </c>
     </row>
@@ -5701,7 +5701,7 @@
       </c>
       <c r="D21" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Correct the reporting period dates to reflect completed, non-future durations.</t>
+          <t xml:space="preserve">Complete the reporting period and refresh annual evidence before independent-verifier handover.</t>
         </is>
       </c>
       <c r="E21" t="inlineStr" s="1">
@@ -5716,7 +5716,7 @@
       </c>
       <c r="G21" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Reporting period dates are valid and complete.</t>
+          <t xml:space="preserve">The reporting period has ended and full-year evidence is complete.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(step8): remove generated report artifacts from scoped fix
</commit_message>
<xml_diff>
--- a/artifacts/sample-v5/Verifier Workspace.xlsx
+++ b/artifacts/sample-v5/Verifier Workspace.xlsx
@@ -4245,12 +4245,12 @@
       </c>
       <c r="E2" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">The structurally complete annual reporting period ends in the future. A conditional operator working file may be generated, but definitive annual readiness and verifier handover remain blocked.</t>
+          <t xml:space="preserve">The reporting period end date is in the future relative to the assessment timestamp. Future periods are blocked from sealing.</t>
         </is>
       </c>
       <c r="F2" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">A future annual period blocks definitive readiness and verifier handover, but not an explicitly conditional operator working file.</t>
+          <t xml:space="preserve">Invalid, future, or incomplete reporting period dates block sealing and readiness.</t>
         </is>
       </c>
     </row>
@@ -5701,7 +5701,7 @@
       </c>
       <c r="D21" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Complete the reporting period and refresh annual evidence before independent-verifier handover.</t>
+          <t xml:space="preserve">Correct the reporting period dates to reflect completed, non-future durations.</t>
         </is>
       </c>
       <c r="E21" t="inlineStr" s="1">
@@ -5716,7 +5716,7 @@
       </c>
       <c r="G21" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">The reporting period has ended and full-year evidence is complete.</t>
+          <t xml:space="preserve">Reporting period dates are valid and complete.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(artifacts): refresh sample-v5 dossiers from evidence quality mapping
Registry template mappings 26/27 now carry MATERIAL_EVIDENCE_QUALITY_D_OR_E
validation and linked evidenceIds, matching the evidence quality semantics
shipped in 01744e2.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/artifacts/sample-v5/Verifier Workspace.xlsx
+++ b/artifacts/sample-v5/Verifier Workspace.xlsx
@@ -4245,12 +4245,12 @@
       </c>
       <c r="E2" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">The reporting period end date is in the future relative to the assessment timestamp. Future periods are blocked from sealing.</t>
+          <t xml:space="preserve">The structurally complete annual reporting period ends in the future. A conditional operator working file may be generated, but definitive annual readiness and verifier handover remain blocked.</t>
         </is>
       </c>
       <c r="F2" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Invalid, future, or incomplete reporting period dates block sealing and readiness.</t>
+          <t xml:space="preserve">A future annual period blocks definitive readiness and verifier handover, but not an explicitly conditional operator working file.</t>
         </is>
       </c>
     </row>
@@ -5701,7 +5701,7 @@
       </c>
       <c r="D21" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Correct the reporting period dates to reflect completed, non-future durations.</t>
+          <t xml:space="preserve">Complete the reporting period and refresh annual evidence before independent-verifier handover.</t>
         </is>
       </c>
       <c r="E21" t="inlineStr" s="1">
@@ -5716,7 +5716,7 @@
       </c>
       <c r="G21" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Reporting period dates are valid and complete.</t>
+          <t xml:space="preserve">The reporting period has ended and full-year evidence is complete.</t>
         </is>
       </c>
     </row>
@@ -5843,7 +5843,7 @@
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Article 6 &amp; Annex</t>
+          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546, Article 6 &amp; Annex</t>
         </is>
       </c>
       <c r="D3" t="inlineStr" s="1">
@@ -5969,7 +5969,7 @@
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Article 6(2)</t>
+          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546, Article 6(2)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr" s="1">
@@ -6132,12 +6132,12 @@
       </c>
       <c r="B10" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">IMPL_2025_2546</t>
+          <t xml:space="preserve">IMPL_2025_2547</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Annex II</t>
+          <t xml:space="preserve">Implementing Regulation (EU) 2025/2547, Article 6 &amp; Annex III</t>
         </is>
       </c>
       <c r="D10" t="inlineStr" s="1">
@@ -6174,12 +6174,12 @@
       </c>
       <c r="B11" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">IMPL_2025_2546</t>
+          <t xml:space="preserve">IMPL_2025_2547</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Annex II.3</t>
+          <t xml:space="preserve">Implementing Regulation (EU) 2025/2547, Annex II</t>
         </is>
       </c>
       <c r="D11" t="inlineStr" s="1">
@@ -6216,12 +6216,12 @@
       </c>
       <c r="B12" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">IMPL_2025_2546</t>
+          <t xml:space="preserve">IMPL_2025_2547</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Annex II.4.1</t>
+          <t xml:space="preserve">Implementing Regulation (EU) 2025/2547, Article 5 &amp; Annex II, point E</t>
         </is>
       </c>
       <c r="D12" t="inlineStr" s="1">
@@ -7710,12 +7710,12 @@
       </c>
       <c r="H28" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">11111111-1111-4111-8111-333333333333</t>
         </is>
       </c>
       <c r="I28" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">REQUIREMENT_NOT_EVALUATED</t>
+          <t xml:space="preserve">MATERIAL_EVIDENCE_QUALITY_D_OR_E | EVIDENCE_DIVERSITY_INSUFFICIENT</t>
         </is>
       </c>
     </row>
@@ -7757,12 +7757,12 @@
       </c>
       <c r="H29" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">11111111-1111-4111-8111-333333333333</t>
         </is>
       </c>
       <c r="I29" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">REQUIREMENT_NOT_EVALUATED</t>
+          <t xml:space="preserve">MATERIAL_EVIDENCE_QUALITY_D_OR_E | EVIDENCE_DIVERSITY_INSUFFICIENT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(artifacts): refresh sample-v5 dossiers from evidence quality mapping (#173)
Registry template mappings 26/27 now carry MATERIAL_EVIDENCE_QUALITY_D_OR_E
validation and linked evidenceIds, matching the evidence quality semantics
shipped in 01744e2.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/artifacts/sample-v5/Verifier Workspace.xlsx
+++ b/artifacts/sample-v5/Verifier Workspace.xlsx
@@ -4245,12 +4245,12 @@
       </c>
       <c r="E2" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">The reporting period end date is in the future relative to the assessment timestamp. Future periods are blocked from sealing.</t>
+          <t xml:space="preserve">The structurally complete annual reporting period ends in the future. A conditional operator working file may be generated, but definitive annual readiness and verifier handover remain blocked.</t>
         </is>
       </c>
       <c r="F2" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Invalid, future, or incomplete reporting period dates block sealing and readiness.</t>
+          <t xml:space="preserve">A future annual period blocks definitive readiness and verifier handover, but not an explicitly conditional operator working file.</t>
         </is>
       </c>
     </row>
@@ -5701,7 +5701,7 @@
       </c>
       <c r="D21" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Correct the reporting period dates to reflect completed, non-future durations.</t>
+          <t xml:space="preserve">Complete the reporting period and refresh annual evidence before independent-verifier handover.</t>
         </is>
       </c>
       <c r="E21" t="inlineStr" s="1">
@@ -5716,7 +5716,7 @@
       </c>
       <c r="G21" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Reporting period dates are valid and complete.</t>
+          <t xml:space="preserve">The reporting period has ended and full-year evidence is complete.</t>
         </is>
       </c>
     </row>
@@ -5843,7 +5843,7 @@
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Article 6 &amp; Annex</t>
+          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546, Article 6 &amp; Annex</t>
         </is>
       </c>
       <c r="D3" t="inlineStr" s="1">
@@ -5969,7 +5969,7 @@
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Article 6(2)</t>
+          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546, Article 6(2)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr" s="1">
@@ -6132,12 +6132,12 @@
       </c>
       <c r="B10" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">IMPL_2025_2546</t>
+          <t xml:space="preserve">IMPL_2025_2547</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Annex II</t>
+          <t xml:space="preserve">Implementing Regulation (EU) 2025/2547, Article 6 &amp; Annex III</t>
         </is>
       </c>
       <c r="D10" t="inlineStr" s="1">
@@ -6174,12 +6174,12 @@
       </c>
       <c r="B11" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">IMPL_2025_2546</t>
+          <t xml:space="preserve">IMPL_2025_2547</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Annex II.3</t>
+          <t xml:space="preserve">Implementing Regulation (EU) 2025/2547, Annex II</t>
         </is>
       </c>
       <c r="D11" t="inlineStr" s="1">
@@ -6216,12 +6216,12 @@
       </c>
       <c r="B12" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">IMPL_2025_2546</t>
+          <t xml:space="preserve">IMPL_2025_2547</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Annex II.4.1</t>
+          <t xml:space="preserve">Implementing Regulation (EU) 2025/2547, Article 5 &amp; Annex II, point E</t>
         </is>
       </c>
       <c r="D12" t="inlineStr" s="1">
@@ -7710,12 +7710,12 @@
       </c>
       <c r="H28" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">11111111-1111-4111-8111-333333333333</t>
         </is>
       </c>
       <c r="I28" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">REQUIREMENT_NOT_EVALUATED</t>
+          <t xml:space="preserve">MATERIAL_EVIDENCE_QUALITY_D_OR_E | EVIDENCE_DIVERSITY_INSUFFICIENT</t>
         </is>
       </c>
     </row>
@@ -7757,12 +7757,12 @@
       </c>
       <c r="H29" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">11111111-1111-4111-8111-333333333333</t>
         </is>
       </c>
       <c r="I29" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">REQUIREMENT_NOT_EVALUATED</t>
+          <t xml:space="preserve">MATERIAL_EVIDENCE_QUALITY_D_OR_E | EVIDENCE_DIVERSITY_INSUFFICIENT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(cbam): production seal pipeline adopts CBAMVALID-DOSSIER-6.0 (RM-CBAMVALID-006)
- seal-service: V6 package-state gate (G-02) replaces the V5 readiness gate;
  NOT_READY removed from the production path; V6 metadata recorded
  (two-axis scores, packageReadinessState, 27-component contract)
- pipeline: Enterprise Compliance Master Record.pdf rendered as the 27th
  component (G-13); releaseContractVersion 6 flows through manifest/contracts
- manifest: CBAMVALID-DOSSIER-6.0 schema with the V6 27-component contract
  (G-05); calculation engine 4.0.0
- master record: control key references the signed manifest record instead of
  embedding the manifest hash (breaks the manifest -> PDF -> manifest cycle)
- types: releaseContractVersion widened to 5|6, releaseVersion cap raised to 6

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/artifacts/sample-v5/Verifier Workspace.xlsx
+++ b/artifacts/sample-v5/Verifier Workspace.xlsx
@@ -347,7 +347,7 @@
       </c>
       <c r="B7" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">9974e21ed553c7a029348d88c16204a5c9107d0f3cf4780eb8f137ab077ee62d</t>
+          <t xml:space="preserve">8fa5dbed0bd33198b3ccd24631f5d824cf231abbdfef62f98a190a6546928c5c</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="4">
@@ -7092,9 +7092,9 @@
           <t xml:space="preserve">OPERATOR</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">COMPLETE_OPERATOR</t>
+      <c r="G15" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">INCOMPLETE_EVIDENCE_MISSING</t>
         </is>
       </c>
       <c r="H15" t="inlineStr" s="1">
@@ -7240,7 +7240,7 @@
       </c>
       <c r="H18" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">11111111-1111-4111-8111-222222222222</t>
         </is>
       </c>
       <c r="I18" t="inlineStr" s="1">
@@ -7287,7 +7287,7 @@
       </c>
       <c r="H19" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">11111111-1111-4111-8111-222222222222</t>
         </is>
       </c>
       <c r="I19" t="inlineStr" s="1">
@@ -7334,7 +7334,7 @@
       </c>
       <c r="H20" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">11111111-1111-4111-8111-222222222222</t>
         </is>
       </c>
       <c r="I20" t="inlineStr" s="1">
@@ -12844,7 +12844,7 @@
       </c>
       <c r="D13" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Calculation root 9974e21ed553c7a029348d88c16204a5c9107d0f3cf4780eb8f137ab077ee62d</t>
+          <t xml:space="preserve">Calculation root 8fa5dbed0bd33198b3ccd24631f5d824cf231abbdfef62f98a190a6546928c5c</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(cbam): refresh sample-v5 dossier artifacts under engine 4.1.0
The V5 sample dossier re-renders with CALCULATION_ENGINE_VERSION 4.1.0
after the v7 engine bump; the produced manifest and signatures are the
new canonical output of the verification-grade pipeline.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/artifacts/sample-v5/Verifier Workspace.xlsx
+++ b/artifacts/sample-v5/Verifier Workspace.xlsx
@@ -347,7 +347,7 @@
       </c>
       <c r="B7" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">8fa5dbed0bd33198b3ccd24631f5d824cf231abbdfef62f98a190a6546928c5c</t>
+          <t xml:space="preserve">1c94a8333f1c71e2bd217e74a1c8ba413c3b5a82615e669175cd2fbd16d38c3e</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="4">
@@ -1144,7 +1144,7 @@
       </c>
       <c r="E2" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">690085cd04f6102b1d2617fa92b671e089632e2db84f8c657a521938be42eb57</t>
+          <t xml:space="preserve">678fdfcd3d2e530cbb5111edac8ecc97b9166353f13a76020e2c3b591e8f6a67</t>
         </is>
       </c>
       <c r="F2" t="inlineStr" s="1">
@@ -1176,7 +1176,7 @@
       </c>
       <c r="E3" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">98a76aac49f58cbd4c0ad68637e03e592b2dd2e0bc7208a8062648de29ffe081</t>
+          <t xml:space="preserve">c6232a73800f3a547c7a12ce6e2c339a65475d5533b317d9e24a652846aa98bf</t>
         </is>
       </c>
       <c r="F3" t="inlineStr" s="1">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="E4" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">a42adefa11c2318ea97772635232793e49b9eea363aa214792981361dd7b5c8f</t>
+          <t xml:space="preserve">3aa55cc59e584262ad8465a63402567eeb119dfbdef646458aba86f066678623</t>
         </is>
       </c>
       <c r="F4" t="inlineStr" s="1">
@@ -1240,7 +1240,7 @@
       </c>
       <c r="E5" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">3bd0d06237ae6b808a635fb731efb40b74fb90a51e42bfe49ed064cb41f03e2f</t>
+          <t xml:space="preserve">7f27fc35a5d967e1aedfa71de63830ede78a9ed2f055949c910dd1550bd4e7ea</t>
         </is>
       </c>
       <c r="F5" t="inlineStr" s="1">
@@ -1272,7 +1272,7 @@
       </c>
       <c r="E6" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">137fc83c1e53a213bd38caccb4359607638050549305b90e340da30d856a26c1</t>
+          <t xml:space="preserve">9b8e198e316018b493f309e90cdb33c7fbcd2dde4cf0381d5d7027fa30b52e60</t>
         </is>
       </c>
       <c r="F6" t="inlineStr" s="1">
@@ -1304,7 +1304,7 @@
       </c>
       <c r="E7" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">2670d4a69b964809495520ced63320b6cced57f17d354d9a422aaf1b7c7df0e9</t>
+          <t xml:space="preserve">396635d6df5529d5cedf7e480a48749f65098a3904e609feaabef12370fb21a5</t>
         </is>
       </c>
       <c r="F7" t="inlineStr" s="1">
@@ -1336,7 +1336,7 @@
       </c>
       <c r="E8" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">1b547bb68197cb8f0357a93b9cd6f8655d4cac8c062d1840050938f4a7d82966</t>
+          <t xml:space="preserve">e0302ee3f4fb777e6b1e70b0a670194f40ca5833ea4698eca3c7254d6de8ed2b</t>
         </is>
       </c>
       <c r="F8" t="inlineStr" s="1">
@@ -1368,7 +1368,7 @@
       </c>
       <c r="E9" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">76091fe6aeb6a241be5e78f0223e8dc69ffda7c5eae1db6c298a6d53f0ab1ce0</t>
+          <t xml:space="preserve">7a08371a15c45394f718657be5baf73e01a63ed555233c0cc93445e0e6983799</t>
         </is>
       </c>
       <c r="F9" t="inlineStr" s="1">
@@ -1400,7 +1400,7 @@
       </c>
       <c r="E10" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">bdc01c46d7eb5638aa74127ef82b89f667474b76860ac46f4849f4233dad1153</t>
+          <t xml:space="preserve">794a3ae67743915f24eb75783c4f327406099a3cdd141cc99b562996e22b5879</t>
         </is>
       </c>
       <c r="F10" t="inlineStr" s="1">
@@ -1432,7 +1432,7 @@
       </c>
       <c r="E11" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">6de700969ce1c750514a4ce1be12d1cac3c5ab0aa49ded70ac630e8cd94ff630</t>
+          <t xml:space="preserve">54570b887ba1203bf11a2084bc218298dd144820b35e409986d0a699df472d82</t>
         </is>
       </c>
       <c r="F11" t="inlineStr" s="1">
@@ -12844,7 +12844,7 @@
       </c>
       <c r="D13" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Calculation root 8fa5dbed0bd33198b3ccd24631f5d824cf231abbdfef62f98a190a6546928c5c</t>
+          <t xml:space="preserve">Calculation root 1c94a8333f1c71e2bd217e74a1c8ba413c3b5a82615e669175cd2fbd16d38c3e</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(gates): resolve G-09 PDF false positive scanning and add humans.txt technical SEO metadata
</commit_message>
<xml_diff>
--- a/artifacts/sample-v5/Verifier Workspace.xlsx
+++ b/artifacts/sample-v5/Verifier Workspace.xlsx
@@ -357,7 +357,7 @@
       </c>
       <c r="D7" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">e6a3338b06245293e69e291c4604861aefc6497021406d94e1d735f9baa46666</t>
+          <t xml:space="preserve">0cf77baf09c681e79d9c8ad738fa66b055df17005662e054c64eb55cae470267</t>
         </is>
       </c>
     </row>
@@ -1700,7 +1700,7 @@
       </c>
       <c r="C4" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Commission Implementing Regulation (EU) 2025/2546 of 10 December 2025 on the application of the principles for verification of declared embedded emissions pursuant to Regulation (EU) 2023/956</t>
+          <t xml:space="preserve">Commission Implementing Regulation (EU) 2025/2546 of 10 December 2025 on the application of the principles for verification of declared embedded emissions pursuant to Regulation (EU) 2023/956 of the European Parliament and of the Council</t>
         </is>
       </c>
       <c r="D4" t="inlineStr" s="9">
@@ -1720,7 +1720,7 @@
       </c>
       <c r="G4" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">reasonable assurance and risk-based verification | 5 percent per-good materiality levels | electronic verification report template | site-visit requirements and waiver conditions | non-conformity and misstatement classification</t>
+          <t xml:space="preserve">definitions of misstatement, materiality level and non-conformity | physical site-visit replacement, virtual visit and waiver conditions | 5 percent per-good materiality levels for embedded emissions and free allocation | electronic verification report template (single Annex)</t>
         </is>
       </c>
     </row>
@@ -1737,7 +1737,7 @@
       </c>
       <c r="C5" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Commission Implementing Regulation (EU) 2025/2547 of 10 December 2025 laying down rules for the application of Regulation (EU) 2023/956 as regards the methods for the calculation of emissions embedded in goods</t>
+          <t xml:space="preserve">Commission Implementing Regulation (EU) 2025/2547 of 10 December 2025 laying down rules for the application of Regulation (EU) 2023/956 of the European Parliament and the Council as regards the methods for the calculation of emissions embedded in goods</t>
         </is>
       </c>
       <c r="D5" t="inlineStr" s="9">
@@ -1757,7 +1757,7 @@
       </c>
       <c r="G5" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">functional units and production processes | monitoring plan minimum elements | sector-specific system boundaries and embedded-emissions methods | default values and actual-value calculation methods</t>
+          <t xml:space="preserve">actual-value system boundaries, production processes and functional units | installation-level monitoring plan and attribution of emissions to goods | default values, alternative defaults and complex-goods precursor rules | operator’s emissions report templates</t>
         </is>
       </c>
     </row>
@@ -1774,7 +1774,7 @@
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Commission Implementing Regulation (EU) 2025/2548 of 10 December 2025 laying down rules for the application of Regulation (EU) 2023/956 as regards the calculation and publication of the price of CBAM certificates</t>
+          <t xml:space="preserve">Commission Implementing Regulation (EU) 2025/2548 of 10 December 2025 laying down rules for the application of Regulation (EU) 2023/956 of the European Parliament and of the Council as regards the calculation and publication of the price of CBAM certificates</t>
         </is>
       </c>
       <c r="D6" t="inlineStr" s="9">
@@ -1794,7 +1794,7 @@
       </c>
       <c r="G6" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">calculation and publication of CBAM certificate prices</t>
+          <t xml:space="preserve">2026 quarterly CBAM certificate price calculation and publication | from 2027 weekly CBAM certificate price calculation and publication</t>
         </is>
       </c>
     </row>
@@ -5843,7 +5843,7 @@
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546, Article 6 &amp; Annex</t>
+          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546, Article 6 and Annex point 1.1</t>
         </is>
       </c>
       <c r="D3" t="inlineStr" s="1">
@@ -5969,7 +5969,7 @@
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546, Article 6(2)</t>
+          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546, Articles 2 to 4 and Annex point 2.2</t>
         </is>
       </c>
       <c r="D6" t="inlineStr" s="1">
@@ -6698,7 +6698,7 @@
       </c>
       <c r="C7" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Article 6 and Annex</t>
+          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Article 6 and Annex point 1.1</t>
         </is>
       </c>
       <c r="D7" t="inlineStr" s="1">
@@ -6745,7 +6745,7 @@
       </c>
       <c r="C8" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Article 6 and Annex</t>
+          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Article 6 and Annex point 1.1</t>
         </is>
       </c>
       <c r="D8" t="inlineStr" s="1">
@@ -6792,7 +6792,7 @@
       </c>
       <c r="C9" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Article 6 and Annex</t>
+          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Article 6 and Annex point 1.1</t>
         </is>
       </c>
       <c r="D9" t="inlineStr" s="1">
@@ -6839,7 +6839,7 @@
       </c>
       <c r="C10" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Article 6 and Annex</t>
+          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Article 6 and Annex point 1.1</t>
         </is>
       </c>
       <c r="D10" t="inlineStr" s="1">
@@ -6886,7 +6886,7 @@
       </c>
       <c r="C11" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Article 6 and Annex</t>
+          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Article 6 and Annex point 1.1</t>
         </is>
       </c>
       <c r="D11" t="inlineStr" s="1">
@@ -6933,7 +6933,7 @@
       </c>
       <c r="C12" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Article 6 and Annex</t>
+          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Article 6 and Annex point 1.1</t>
         </is>
       </c>
       <c r="D12" t="inlineStr" s="1">
@@ -6980,7 +6980,7 @@
       </c>
       <c r="C13" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Article 6 and Annex</t>
+          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Article 6 and Annex point 1.1</t>
         </is>
       </c>
       <c r="D13" t="inlineStr" s="1">
@@ -7027,7 +7027,7 @@
       </c>
       <c r="C14" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Article 6 and Annex</t>
+          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Article 6 and Annex point 1.1</t>
         </is>
       </c>
       <c r="D14" t="inlineStr" s="1">
@@ -7074,7 +7074,7 @@
       </c>
       <c r="C15" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Article 6 and Annex</t>
+          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Article 6 and Annex point 1.1</t>
         </is>
       </c>
       <c r="D15" t="inlineStr" s="1">
@@ -7121,7 +7121,7 @@
       </c>
       <c r="C16" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Article 6 and Annex</t>
+          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Article 6 and Annex point 1.1</t>
         </is>
       </c>
       <c r="D16" t="inlineStr" s="1">
@@ -7168,7 +7168,7 @@
       </c>
       <c r="C17" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Article 6 and Annex</t>
+          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Article 6 and Annex point 1.1</t>
         </is>
       </c>
       <c r="D17" t="inlineStr" s="1">
@@ -7450,7 +7450,7 @@
       </c>
       <c r="C23" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Annex II</t>
+          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Article 6 and Annex point 2.4</t>
         </is>
       </c>
       <c r="D23" t="inlineStr" s="1">
@@ -7591,7 +7591,7 @@
       </c>
       <c r="C26" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Annex II</t>
+          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Article 6 and Annex point 2.4</t>
         </is>
       </c>
       <c r="D26" t="inlineStr" s="1">
@@ -7685,7 +7685,7 @@
       </c>
       <c r="C28" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Article 6(3)</t>
+          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Article 6 and Annex point 2.4</t>
         </is>
       </c>
       <c r="D28" t="inlineStr" s="1">
@@ -7732,7 +7732,7 @@
       </c>
       <c r="C29" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Article 6(3)</t>
+          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Article 6 and Annex point 2.4</t>
         </is>
       </c>
       <c r="D29" t="inlineStr" s="1">
@@ -7779,7 +7779,7 @@
       </c>
       <c r="C30" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Annex II.4</t>
+          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Article 6 and Annex point 2.5</t>
         </is>
       </c>
       <c r="D30" t="inlineStr" s="1">
@@ -7826,7 +7826,7 @@
       </c>
       <c r="C31" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Annex II</t>
+          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Article 6 and Annex point 2.4</t>
         </is>
       </c>
       <c r="D31" t="inlineStr" s="1">
@@ -8202,7 +8202,7 @@
       </c>
       <c r="C39" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Article 6(2)</t>
+          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Articles 2 to 4 and Annex point 2.2</t>
         </is>
       </c>
       <c r="D39" t="inlineStr" s="1">
@@ -8249,7 +8249,7 @@
       </c>
       <c r="C40" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Article 6(2)</t>
+          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Articles 2 to 4 and Annex point 2.2</t>
         </is>
       </c>
       <c r="D40" t="inlineStr" s="1">

</xml_diff>

<commit_message>
fix(seo): technical SEO indexing audit & G-09 release gate fix (#283)
* seo: technical seo and indexing audit refinements for canonical urls and indexnow key

* fix(gates): resolve G-09 PDF false positive scanning and add humans.txt technical SEO metadata
</commit_message>
<xml_diff>
--- a/artifacts/sample-v5/Verifier Workspace.xlsx
+++ b/artifacts/sample-v5/Verifier Workspace.xlsx
@@ -357,7 +357,7 @@
       </c>
       <c r="D7" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">e6a3338b06245293e69e291c4604861aefc6497021406d94e1d735f9baa46666</t>
+          <t xml:space="preserve">0cf77baf09c681e79d9c8ad738fa66b055df17005662e054c64eb55cae470267</t>
         </is>
       </c>
     </row>
@@ -1700,7 +1700,7 @@
       </c>
       <c r="C4" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Commission Implementing Regulation (EU) 2025/2546 of 10 December 2025 on the application of the principles for verification of declared embedded emissions pursuant to Regulation (EU) 2023/956</t>
+          <t xml:space="preserve">Commission Implementing Regulation (EU) 2025/2546 of 10 December 2025 on the application of the principles for verification of declared embedded emissions pursuant to Regulation (EU) 2023/956 of the European Parliament and of the Council</t>
         </is>
       </c>
       <c r="D4" t="inlineStr" s="9">
@@ -1720,7 +1720,7 @@
       </c>
       <c r="G4" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">reasonable assurance and risk-based verification | 5 percent per-good materiality levels | electronic verification report template | site-visit requirements and waiver conditions | non-conformity and misstatement classification</t>
+          <t xml:space="preserve">definitions of misstatement, materiality level and non-conformity | physical site-visit replacement, virtual visit and waiver conditions | 5 percent per-good materiality levels for embedded emissions and free allocation | electronic verification report template (single Annex)</t>
         </is>
       </c>
     </row>
@@ -1737,7 +1737,7 @@
       </c>
       <c r="C5" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Commission Implementing Regulation (EU) 2025/2547 of 10 December 2025 laying down rules for the application of Regulation (EU) 2023/956 as regards the methods for the calculation of emissions embedded in goods</t>
+          <t xml:space="preserve">Commission Implementing Regulation (EU) 2025/2547 of 10 December 2025 laying down rules for the application of Regulation (EU) 2023/956 of the European Parliament and the Council as regards the methods for the calculation of emissions embedded in goods</t>
         </is>
       </c>
       <c r="D5" t="inlineStr" s="9">
@@ -1757,7 +1757,7 @@
       </c>
       <c r="G5" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">functional units and production processes | monitoring plan minimum elements | sector-specific system boundaries and embedded-emissions methods | default values and actual-value calculation methods</t>
+          <t xml:space="preserve">actual-value system boundaries, production processes and functional units | installation-level monitoring plan and attribution of emissions to goods | default values, alternative defaults and complex-goods precursor rules | operator’s emissions report templates</t>
         </is>
       </c>
     </row>
@@ -1774,7 +1774,7 @@
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Commission Implementing Regulation (EU) 2025/2548 of 10 December 2025 laying down rules for the application of Regulation (EU) 2023/956 as regards the calculation and publication of the price of CBAM certificates</t>
+          <t xml:space="preserve">Commission Implementing Regulation (EU) 2025/2548 of 10 December 2025 laying down rules for the application of Regulation (EU) 2023/956 of the European Parliament and of the Council as regards the calculation and publication of the price of CBAM certificates</t>
         </is>
       </c>
       <c r="D6" t="inlineStr" s="9">
@@ -1794,7 +1794,7 @@
       </c>
       <c r="G6" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">calculation and publication of CBAM certificate prices</t>
+          <t xml:space="preserve">2026 quarterly CBAM certificate price calculation and publication | from 2027 weekly CBAM certificate price calculation and publication</t>
         </is>
       </c>
     </row>
@@ -5843,7 +5843,7 @@
       </c>
       <c r="C3" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546, Article 6 &amp; Annex</t>
+          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546, Article 6 and Annex point 1.1</t>
         </is>
       </c>
       <c r="D3" t="inlineStr" s="1">
@@ -5969,7 +5969,7 @@
       </c>
       <c r="C6" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546, Article 6(2)</t>
+          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546, Articles 2 to 4 and Annex point 2.2</t>
         </is>
       </c>
       <c r="D6" t="inlineStr" s="1">
@@ -6698,7 +6698,7 @@
       </c>
       <c r="C7" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Article 6 and Annex</t>
+          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Article 6 and Annex point 1.1</t>
         </is>
       </c>
       <c r="D7" t="inlineStr" s="1">
@@ -6745,7 +6745,7 @@
       </c>
       <c r="C8" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Article 6 and Annex</t>
+          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Article 6 and Annex point 1.1</t>
         </is>
       </c>
       <c r="D8" t="inlineStr" s="1">
@@ -6792,7 +6792,7 @@
       </c>
       <c r="C9" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Article 6 and Annex</t>
+          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Article 6 and Annex point 1.1</t>
         </is>
       </c>
       <c r="D9" t="inlineStr" s="1">
@@ -6839,7 +6839,7 @@
       </c>
       <c r="C10" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Article 6 and Annex</t>
+          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Article 6 and Annex point 1.1</t>
         </is>
       </c>
       <c r="D10" t="inlineStr" s="1">
@@ -6886,7 +6886,7 @@
       </c>
       <c r="C11" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Article 6 and Annex</t>
+          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Article 6 and Annex point 1.1</t>
         </is>
       </c>
       <c r="D11" t="inlineStr" s="1">
@@ -6933,7 +6933,7 @@
       </c>
       <c r="C12" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Article 6 and Annex</t>
+          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Article 6 and Annex point 1.1</t>
         </is>
       </c>
       <c r="D12" t="inlineStr" s="1">
@@ -6980,7 +6980,7 @@
       </c>
       <c r="C13" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Article 6 and Annex</t>
+          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Article 6 and Annex point 1.1</t>
         </is>
       </c>
       <c r="D13" t="inlineStr" s="1">
@@ -7027,7 +7027,7 @@
       </c>
       <c r="C14" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Article 6 and Annex</t>
+          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Article 6 and Annex point 1.1</t>
         </is>
       </c>
       <c r="D14" t="inlineStr" s="1">
@@ -7074,7 +7074,7 @@
       </c>
       <c r="C15" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Article 6 and Annex</t>
+          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Article 6 and Annex point 1.1</t>
         </is>
       </c>
       <c r="D15" t="inlineStr" s="1">
@@ -7121,7 +7121,7 @@
       </c>
       <c r="C16" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Article 6 and Annex</t>
+          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Article 6 and Annex point 1.1</t>
         </is>
       </c>
       <c r="D16" t="inlineStr" s="1">
@@ -7168,7 +7168,7 @@
       </c>
       <c r="C17" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Article 6 and Annex</t>
+          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Article 6 and Annex point 1.1</t>
         </is>
       </c>
       <c r="D17" t="inlineStr" s="1">
@@ -7450,7 +7450,7 @@
       </c>
       <c r="C23" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Annex II</t>
+          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Article 6 and Annex point 2.4</t>
         </is>
       </c>
       <c r="D23" t="inlineStr" s="1">
@@ -7591,7 +7591,7 @@
       </c>
       <c r="C26" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Annex II</t>
+          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Article 6 and Annex point 2.4</t>
         </is>
       </c>
       <c r="D26" t="inlineStr" s="1">
@@ -7685,7 +7685,7 @@
       </c>
       <c r="C28" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Article 6(3)</t>
+          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Article 6 and Annex point 2.4</t>
         </is>
       </c>
       <c r="D28" t="inlineStr" s="1">
@@ -7732,7 +7732,7 @@
       </c>
       <c r="C29" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Article 6(3)</t>
+          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Article 6 and Annex point 2.4</t>
         </is>
       </c>
       <c r="D29" t="inlineStr" s="1">
@@ -7779,7 +7779,7 @@
       </c>
       <c r="C30" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Annex II.4</t>
+          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Article 6 and Annex point 2.5</t>
         </is>
       </c>
       <c r="D30" t="inlineStr" s="1">
@@ -7826,7 +7826,7 @@
       </c>
       <c r="C31" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Annex II</t>
+          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Article 6 and Annex point 2.4</t>
         </is>
       </c>
       <c r="D31" t="inlineStr" s="1">
@@ -8202,7 +8202,7 @@
       </c>
       <c r="C39" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Article 6(2)</t>
+          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Articles 2 to 4 and Annex point 2.2</t>
         </is>
       </c>
       <c r="D39" t="inlineStr" s="1">
@@ -8249,7 +8249,7 @@
       </c>
       <c r="C40" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Article 6(2)</t>
+          <t xml:space="preserve">Implementing Regulation (EU) 2025/2546 Articles 2 to 4 and Annex point 2.2</t>
         </is>
       </c>
       <c r="D40" t="inlineStr" s="1">

</xml_diff>